<commit_message>
docs: add and update rehearsal checklists
</commit_message>
<xml_diff>
--- a/docs/rehearsal/checklist.xlsx
+++ b/docs/rehearsal/checklist.xlsx
@@ -26,12 +26,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1400" uniqueCount="761">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1402" uniqueCount="763">
   <si>
     <t xml:space="preserve">StayGuard: checklist diễn tập (Gate 1)</t>
   </si>
   <si>
-    <t xml:space="preserve">Cập nhật 03/10/2026 tối. Phạm vi: demo portfolio, không có khách thật; các dòng cần nhà nghỉ thật, tiền thật hoặc hạ tầng thật là Bỏ qua kèm lý do. Kết quả tự động (QA, make demo-check) ghi Đạt kèm ghi chú 'QA tự động &lt;ngày&gt;'; các dòng cần mắt người (GD-03 đến GD-07, TD-05, TD-08) chỉ nhận ghi chú và chờ bạn xem. TT-21, TT-22, TT-26 giữ Chờ thử lại vì test chưa phủ hết kỳ vọng. Đã gộp GL-13 đến GL-16 của phiên khác; các dòng trùng mã đã gỡ.</t>
+    <t xml:space="preserve">Cập nhật 03/10/2026 tối. Phạm vi: demo portfolio, không có khách thật; các dòng cần nhà nghỉ thật, tiền thật hoặc hạ tầng thật là Bỏ qua kèm lý do. Kết quả tự động (QA, make demo-check) ghi Đạt kèm ghi chú 'QA tự động &lt;ngày&gt;'; các dòng cần mắt người (GD-03 đến GD-07, TD-05, TD-08) chỉ nhận ghi chú và chờ bạn xem. TT-21, TT-22, TT-26 giữ Chờ thử lại vì test chưa phủ hết kỳ vọng. Đã gộp GL-13 đến GL-16 của phiên khác; các dòng trùng mã đã gỡ. Cập nhật 04/10/2026: make demo-check xanh 8/8 và CI GitHub xanh 9/9 (run #243).</t>
   </si>
   <si>
     <t xml:space="preserve">Cách dùng</t>
@@ -311,7 +311,8 @@
     <t xml:space="preserve">Cao</t>
   </si>
   <si>
-    <t xml:space="preserve">Số test đã tăng: make smoke hiện chạy 9 spec (WEB-1 báo 9 passed trên máy của lane, chưa phải bạn). Cập nhật kỳ vọng khi bạn thử.</t>
+    <t xml:space="preserve">Số test đã tăng: make smoke hiện chạy 9 spec (WEB-1 báo 9 passed trên máy của lane, chưa phải bạn). Cập nhật kỳ vọng khi bạn thử.
+make smoke xanh trong make demo-check (04/10/2026, QA tự động); nay chạy 10 spec.</t>
   </si>
   <si>
     <t xml:space="preserve">CB-02</t>
@@ -710,7 +711,8 @@
     <t xml:space="preserve">Màn tự hiện QR hết hạn, có nút tạo QR mới. Tiền chuyển vào mã cũ vẫn được ghi nhận khi SePay báo.</t>
   </si>
   <si>
-    <t xml:space="preserve">QA tự động 03/10/2026. QR không bao giờ chuyển EXPIRED theo thời gian: ExpirePending chỉ chạy khi tạo thanh toán mới, qrExpiryMinutes chỉ được lưu. Đề xuất: suy ra EXPIRED lúc đọc, giữ bản ghi PENDING để tiền về mã cũ vẫn khớp. Giao API-2.</t>
+    <t xml:space="preserve">QA tự động 03/10/2026. QR không bao giờ chuyển EXPIRED theo thời gian: ExpirePending chỉ chạy khi tạo thanh toán mới, qrExpiryMinutes chỉ được lưu. Đề xuất: suy ra EXPIRED lúc đọc, giữ bản ghi PENDING để tiền về mã cũ vẫn khớp. Giao API-2.
+QA tự động 04/10/2026: QR quá hạn trả EXPIRED (e640f86, suy ra lúc đọc), tiền về mã cũ vẫn khớp; e2e smoke.then-expiry của WEB-1 đạt, demo-check xanh.</t>
   </si>
   <si>
     <t xml:space="preserve">TT-16</t>
@@ -807,7 +809,8 @@
   <si>
     <t xml:space="preserve">03/10 08:48: A102 bị kẹt, ô phòng mất loại thuê và giờ ở, không bấm vào được.
 Đã sửa một phần (WEB-1 f6add89): ô Chờ hoàn ₫X và nút Hoàn lại khách khi mở lại. Mới có unit test, chưa chạy với hoàn cọc thật. Thử lại sau rebuild.
-QA tự động đạt. Giữ Chờ thử lại vì kỳ vọng có 'dữ liệu cũ cũng xử lý được', test dùng nhà nghỉ mới.</t>
+QA tự động đạt. Giữ Chờ thử lại vì kỳ vọng có 'dữ liệu cũ cũng xử lý được', test dùng nhà nghỉ mới.
+demo-check 04/10 xanh. Vẫn chờ bạn thử với dữ liệu cũ.</t>
   </si>
   <si>
     <t xml:space="preserve">TT-22</t>
@@ -824,7 +827,8 @@
   <si>
     <t xml:space="preserve">API-2 phải trả lời: giờ ra chốt lúc mở màn hay lúc xác nhận thanh toán.
 WEB-1 báo API chốt giờ ra lúc xác nhận thanh toán (rời màn mà chưa xác nhận thì lượt vẫn đang ở). Cần xác nhận lại với API-2 rồi thử tay.
-QA tự động đạt. Giữ Chờ thử lại cho tới khi API-2 xác nhận quy tắc giờ ra (WEB-1 báo: chốt lúc xác nhận thanh toán).</t>
+QA tự động đạt. Giữ Chờ thử lại cho tới khi API-2 xác nhận quy tắc giờ ra (WEB-1 báo: chốt lúc xác nhận thanh toán).
+demo-check 04/10 xanh. Vẫn chờ API-2 xác nhận quy tắc giờ ra.</t>
   </si>
   <si>
     <t xml:space="preserve">TT-23</t>
@@ -889,7 +893,8 @@
   </si>
   <si>
     <t xml:space="preserve">03/10 08:42: A101 ghi cọc 0đ, phải thu 80.000đ. API-2 đối chiếu cọc lúc đọc và sửa dữ liệu cũ; WEB-1 đọc đúng trường. Gốc rễ chưa tái hiện được.
-QA tự động đạt trên nhà nghỉ mới. Gốc rễ ban đầu chưa tái hiện được nên giữ Chờ thử lại cho tới khi bạn mở lại màn trả phòng trên dữ liệu của bạn.</t>
+QA tự động đạt trên nhà nghỉ mới. Gốc rễ ban đầu chưa tái hiện được nên giữ Chờ thử lại cho tới khi bạn mở lại màn trả phòng trên dữ liệu của bạn.
+demo-check 04/10 xanh sau khi sửa test (đọc đúng dòng cọc; ảnh chụp thấy cọc ₫250,000). Vẫn chờ bạn mở lại màn trả phòng trên dữ liệu của bạn.</t>
   </si>
   <si>
     <t xml:space="preserve">TT-27</t>
@@ -1054,7 +1059,8 @@
     <t xml:space="preserve">Thấy số đếm, khoản chi, lý do, người bàn giao.</t>
   </si>
   <si>
-    <t xml:space="preserve">QA tự động 03/10/2026. Màn đối soát ca không nêu người bàn giao. Đề xuất: người đóng ca (tên, vai trò) và quỹ để lại; hệ thống không có người nhận ca. Giao API-2 và WEB-2.</t>
+    <t xml:space="preserve">QA tự động 03/10/2026. Màn đối soát ca không nêu người bàn giao. Đề xuất: người đóng ca (tên, vai trò) và quỹ để lại; hệ thống không có người nhận ca. Giao API-2 và WEB-2.
+04/10/2026: API trả closedByName, closedByRole, floatLeft (318d2a0, 3214b9d); màn Đối soát ca có Người bàn giao và Để lại két (WEB-2). QA tự động đạt. Chưa xem màn trên API thật: bạn mở Đối soát ca một lần rồi chuyển Đạt.</t>
   </si>
   <si>
     <t xml:space="preserve">CA-09</t>
@@ -1975,6 +1981,9 @@
     <t xml:space="preserve">Xanh. Gồm chữ ký, thời gian, chống trùng, giao dịch tiền ra.</t>
   </si>
   <si>
+    <t xml:space="preserve">Bộ test webhook tự động là make test-api-int: xanh trong demo-check và trên CI #243 (04/10/2026).</t>
+  </si>
+  <si>
     <t xml:space="preserve">VH-01</t>
   </si>
   <si>
@@ -2169,6 +2178,9 @@
   </si>
   <si>
     <t xml:space="preserve">Cả 8 kiểm tra xanh: checks, lint, contracts, licenses, secrets, test-api, test-api-int, test-web.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI xanh 9/9 job (run #243, commit 92472f7, 04/10/2026): lint, checks, test-api, test-api-int, test-web, contracts, image, secrets, licenses. Repo public.</t>
   </si>
   <si>
     <t xml:space="preserve">GL-02</t>
@@ -2784,7 +2796,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="24">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -2934,14 +2946,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFE0DED8"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF5C2BD"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -3564,7 +3568,7 @@
       </c>
       <c r="C5" s="9" t="n">
         <f aca="false">COUNTIFS(Checklist!$B$2:$B$300,$A5,Checklist!$H$2:$H$300,"Đạt")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D5" s="9" t="n">
         <f aca="false">COUNTIFS(Checklist!$B$2:$B$300,$A5,Checklist!$H$2:$H$300,"Lỗi")</f>
@@ -3580,11 +3584,11 @@
       </c>
       <c r="G5" s="9" t="n">
         <f aca="false">B5-C5-D5-E5-F5</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H5" s="10" t="n">
         <f aca="false">IFERROR(C5/(B5-F5),0)</f>
-        <v>0.625</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3597,11 +3601,11 @@
       </c>
       <c r="C6" s="9" t="n">
         <f aca="false">COUNTIFS(Checklist!$B$2:$B$300,$A6,Checklist!$H$2:$H$300,"Đạt")</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6" s="9" t="n">
         <f aca="false">COUNTIFS(Checklist!$B$2:$B$300,$A6,Checklist!$H$2:$H$300,"Lỗi")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="9" t="n">
         <f aca="false">COUNTIFS(Checklist!$B$2:$B$300,$A6,Checklist!$H$2:$H$300,"Chờ thử lại")</f>
@@ -3617,7 +3621,7 @@
       </c>
       <c r="H6" s="10" t="n">
         <f aca="false">IFERROR(C6/(B6-F6),0)</f>
-        <v>0.851851851851852</v>
+        <v>0.888888888888889</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3634,11 +3638,11 @@
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">COUNTIFS(Checklist!$B$2:$B$300,$A7,Checklist!$H$2:$H$300,"Lỗi")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">COUNTIFS(Checklist!$B$2:$B$300,$A7,Checklist!$H$2:$H$300,"Chờ thử lại")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" s="9" t="n">
         <f aca="false">COUNTIFS(Checklist!$B$2:$B$300,$A7,Checklist!$H$2:$H$300,"Bỏ qua")</f>
@@ -3861,7 +3865,7 @@
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">COUNTIFS(Checklist!$B$2:$B$300,$A14,Checklist!$H$2:$H$300,"Đạt")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">COUNTIFS(Checklist!$B$2:$B$300,$A14,Checklist!$H$2:$H$300,"Lỗi")</f>
@@ -3877,11 +3881,11 @@
       </c>
       <c r="G14" s="9" t="n">
         <f aca="false">B14-C14-D14-E14-F14</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14" s="10" t="n">
         <f aca="false">IFERROR(C14/(B14-F14),0)</f>
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3960,7 +3964,7 @@
       </c>
       <c r="C17" s="9" t="n">
         <f aca="false">COUNTIFS(Checklist!$B$2:$B$300,$A17,Checklist!$H$2:$H$300,"Đạt")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="9" t="n">
         <f aca="false">COUNTIFS(Checklist!$B$2:$B$300,$A17,Checklist!$H$2:$H$300,"Lỗi")</f>
@@ -3976,11 +3980,11 @@
       </c>
       <c r="G17" s="9" t="n">
         <f aca="false">B17-C17-D17-E17-F17</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H17" s="10" t="n">
         <f aca="false">IFERROR(C17/(B17-F17),0)</f>
-        <v>0</v>
+        <v>0.166666666666667</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3993,15 +3997,15 @@
       </c>
       <c r="C18" s="18" t="n">
         <f aca="false">SUM(C5:C17)</f>
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D18" s="18" t="n">
         <f aca="false">SUM(D5:D17)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E18" s="18" t="n">
         <f aca="false">SUM(E5:E17)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F18" s="18" t="n">
         <f aca="false">SUM(F5:F17)</f>
@@ -4009,11 +4013,11 @@
       </c>
       <c r="G18" s="18" t="n">
         <f aca="false">SUM(G5:G17)</f>
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H18" s="19" t="n">
         <f aca="false">IFERROR(C18/(B18-F18),0)</f>
-        <v>0.795275590551181</v>
+        <v>0.826771653543307</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4027,7 +4031,7 @@
       </c>
       <c r="B21" s="21" t="n">
         <f aca="false">COUNTIFS(Checklist!$G$2:$G$300,"Cao")-COUNTIFS(Checklist!$G$2:$G$300,"Cao",Checklist!$H$2:$H$300,"Đạt")-COUNTIFS(Checklist!$G$2:$G$300,"Cao",Checklist!$H$2:$H$300,"Bỏ qua")</f>
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4036,7 +4040,7 @@
       </c>
       <c r="B22" s="21" t="n">
         <f aca="false">D18</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4168,9 +4172,11 @@
         <v>93</v>
       </c>
       <c r="H2" s="31" t="s">
-        <v>61</v>
-      </c>
-      <c r="I2" s="32"/>
+        <v>12</v>
+      </c>
+      <c r="I2" s="32" t="n">
+        <v>46299</v>
+      </c>
       <c r="J2" s="33" t="s">
         <v>94</v>
       </c>
@@ -4952,10 +4958,10 @@
         <v>134</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="I27" s="32" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="J27" s="33" t="s">
         <v>219</v>
@@ -5646,11 +5652,9 @@
         <v>134</v>
       </c>
       <c r="H49" s="31" t="s">
-        <v>58</v>
-      </c>
-      <c r="I49" s="32" t="n">
-        <v>46298</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="I49" s="32"/>
       <c r="J49" s="33" t="s">
         <v>325</v>
       </c>
@@ -7812,14 +7816,18 @@
         <v>93</v>
       </c>
       <c r="H117" s="31" t="s">
-        <v>61</v>
-      </c>
-      <c r="I117" s="32"/>
-      <c r="J117" s="33"/>
+        <v>12</v>
+      </c>
+      <c r="I117" s="32" t="n">
+        <v>46299</v>
+      </c>
+      <c r="J117" s="33" t="s">
+        <v>621</v>
+      </c>
     </row>
     <row r="118" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="26" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B118" s="27" t="s">
         <v>73</v>
@@ -7828,13 +7836,13 @@
         <v>89</v>
       </c>
       <c r="D118" s="29" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="E118" s="28" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="F118" s="28" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="G118" s="30" t="s">
         <v>93</v>
@@ -7844,12 +7852,12 @@
       </c>
       <c r="I118" s="32"/>
       <c r="J118" s="33" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="26" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B119" s="27" t="s">
         <v>73</v>
@@ -7858,13 +7866,13 @@
         <v>89</v>
       </c>
       <c r="D119" s="29" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="E119" s="28" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="F119" s="28" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="G119" s="30" t="s">
         <v>134</v>
@@ -7881,7 +7889,7 @@
     </row>
     <row r="120" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="26" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="B120" s="27" t="s">
         <v>73</v>
@@ -7890,13 +7898,13 @@
         <v>89</v>
       </c>
       <c r="D120" s="29" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="E120" s="28" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="F120" s="28" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="G120" s="30" t="s">
         <v>93</v>
@@ -7908,12 +7916,12 @@
         <v>46298</v>
       </c>
       <c r="J120" s="33" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="26" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B121" s="27" t="s">
         <v>73</v>
@@ -7922,13 +7930,13 @@
         <v>89</v>
       </c>
       <c r="D121" s="29" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="E121" s="28" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="F121" s="28" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G121" s="30" t="s">
         <v>93</v>
@@ -7938,12 +7946,12 @@
       </c>
       <c r="I121" s="32"/>
       <c r="J121" s="33" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="26" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B122" s="27" t="s">
         <v>73</v>
@@ -7952,13 +7960,13 @@
         <v>89</v>
       </c>
       <c r="D122" s="29" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E122" s="28" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="F122" s="28" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="G122" s="30" t="s">
         <v>93</v>
@@ -7975,7 +7983,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="26" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B123" s="27" t="s">
         <v>73</v>
@@ -7984,13 +7992,13 @@
         <v>89</v>
       </c>
       <c r="D123" s="29" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="E123" s="28" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="F123" s="28" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="G123" s="30" t="s">
         <v>134</v>
@@ -8007,7 +8015,7 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="26" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B124" s="27" t="s">
         <v>73</v>
@@ -8016,13 +8024,13 @@
         <v>89</v>
       </c>
       <c r="D124" s="29" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="E124" s="28" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="F124" s="28" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="G124" s="30" t="s">
         <v>145</v>
@@ -8032,12 +8040,12 @@
       </c>
       <c r="I124" s="32"/>
       <c r="J124" s="33" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="26" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B125" s="35" t="s">
         <v>74</v>
@@ -8046,13 +8054,13 @@
         <v>169</v>
       </c>
       <c r="D125" s="29" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="E125" s="28" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="F125" s="28" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="G125" s="30" t="s">
         <v>93</v>
@@ -8065,7 +8073,7 @@
     </row>
     <row r="126" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="26" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B126" s="35" t="s">
         <v>74</v>
@@ -8074,13 +8082,13 @@
         <v>141</v>
       </c>
       <c r="D126" s="29" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="E126" s="28" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="F126" s="28" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="G126" s="30" t="s">
         <v>134</v>
@@ -8093,7 +8101,7 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="26" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B127" s="35" t="s">
         <v>74</v>
@@ -8102,13 +8110,13 @@
         <v>141</v>
       </c>
       <c r="D127" s="29" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="E127" s="28" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="F127" s="28" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="G127" s="30" t="s">
         <v>134</v>
@@ -8123,7 +8131,7 @@
     </row>
     <row r="128" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="26" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B128" s="35" t="s">
         <v>74</v>
@@ -8132,13 +8140,13 @@
         <v>141</v>
       </c>
       <c r="D128" s="29" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="E128" s="28" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="F128" s="28" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="G128" s="30" t="s">
         <v>134</v>
@@ -8153,7 +8161,7 @@
     </row>
     <row r="129" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="26" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B129" s="35" t="s">
         <v>74</v>
@@ -8162,13 +8170,13 @@
         <v>169</v>
       </c>
       <c r="D129" s="29" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="E129" s="28" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="F129" s="28" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="G129" s="30" t="s">
         <v>134</v>
@@ -8183,7 +8191,7 @@
     </row>
     <row r="130" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="26" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B130" s="35" t="s">
         <v>74</v>
@@ -8192,13 +8200,13 @@
         <v>130</v>
       </c>
       <c r="D130" s="29" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="E130" s="28" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="F130" s="28" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="G130" s="30" t="s">
         <v>134</v>
@@ -8213,7 +8221,7 @@
     </row>
     <row r="131" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="26" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B131" s="35" t="s">
         <v>74</v>
@@ -8222,13 +8230,13 @@
         <v>169</v>
       </c>
       <c r="D131" s="29" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="E131" s="28" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="F131" s="28" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="G131" s="30" t="s">
         <v>145</v>
@@ -8243,7 +8251,7 @@
     </row>
     <row r="132" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="26" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="B132" s="37" t="s">
         <v>75</v>
@@ -8252,26 +8260,30 @@
         <v>89</v>
       </c>
       <c r="D132" s="29" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="E132" s="28" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="F132" s="28" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="G132" s="30" t="s">
         <v>93</v>
       </c>
       <c r="H132" s="31" t="s">
-        <v>61</v>
-      </c>
-      <c r="I132" s="32"/>
-      <c r="J132" s="33"/>
+        <v>12</v>
+      </c>
+      <c r="I132" s="32" t="n">
+        <v>46299</v>
+      </c>
+      <c r="J132" s="33" t="s">
+        <v>686</v>
+      </c>
     </row>
     <row r="133" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="26" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="B133" s="37" t="s">
         <v>75</v>
@@ -8280,13 +8292,13 @@
         <v>89</v>
       </c>
       <c r="D133" s="29" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="E133" s="28" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="F133" s="28" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="G133" s="30" t="s">
         <v>93</v>
@@ -8296,12 +8308,12 @@
       </c>
       <c r="I133" s="32"/>
       <c r="J133" s="33" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="26" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="B134" s="37" t="s">
         <v>75</v>
@@ -8310,13 +8322,13 @@
         <v>89</v>
       </c>
       <c r="D134" s="29" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="E134" s="28" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="F134" s="28" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="G134" s="30" t="s">
         <v>93</v>
@@ -8326,12 +8338,12 @@
       </c>
       <c r="I134" s="32"/>
       <c r="J134" s="33" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="26" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="B135" s="37" t="s">
         <v>75</v>
@@ -8340,13 +8352,13 @@
         <v>280</v>
       </c>
       <c r="D135" s="29" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="E135" s="28" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="F135" s="28" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="G135" s="30" t="s">
         <v>93</v>
@@ -8356,12 +8368,12 @@
       </c>
       <c r="I135" s="32"/>
       <c r="J135" s="33" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="26" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B136" s="37" t="s">
         <v>75</v>
@@ -8370,13 +8382,13 @@
         <v>89</v>
       </c>
       <c r="D136" s="29" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="E136" s="28" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="F136" s="28" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="G136" s="30" t="s">
         <v>93</v>
@@ -8386,12 +8398,12 @@
       </c>
       <c r="I136" s="32"/>
       <c r="J136" s="33" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="26" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="B137" s="37" t="s">
         <v>75</v>
@@ -8400,13 +8412,13 @@
         <v>280</v>
       </c>
       <c r="D137" s="29" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="E137" s="28" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="F137" s="28" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G137" s="30" t="s">
         <v>93</v>
@@ -8416,12 +8428,12 @@
       </c>
       <c r="I137" s="32"/>
       <c r="J137" s="33" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="26" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B138" s="37" t="s">
         <v>75</v>
@@ -8430,13 +8442,13 @@
         <v>89</v>
       </c>
       <c r="D138" s="29" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="E138" s="28" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="F138" s="28" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="G138" s="30" t="s">
         <v>93</v>
@@ -8446,12 +8458,12 @@
       </c>
       <c r="I138" s="32"/>
       <c r="J138" s="33" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="26" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="B139" s="37" t="s">
         <v>75</v>
@@ -8460,13 +8472,13 @@
         <v>89</v>
       </c>
       <c r="D139" s="29" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="E139" s="28" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="F139" s="28" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="G139" s="30" t="s">
         <v>93</v>
@@ -8476,12 +8488,12 @@
       </c>
       <c r="I139" s="32"/>
       <c r="J139" s="33" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="26" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="B140" s="37" t="s">
         <v>75</v>
@@ -8490,13 +8502,13 @@
         <v>141</v>
       </c>
       <c r="D140" s="29" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="E140" s="28" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="F140" s="28" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="G140" s="30" t="s">
         <v>93</v>
@@ -8506,27 +8518,27 @@
       </c>
       <c r="I140" s="32"/>
       <c r="J140" s="33" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="26" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B141" s="37" t="s">
         <v>75</v>
       </c>
       <c r="C141" s="28" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="D141" s="29" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="E141" s="28" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="F141" s="28" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="G141" s="30" t="s">
         <v>93</v>
@@ -8536,12 +8548,12 @@
       </c>
       <c r="I141" s="32"/>
       <c r="J141" s="33" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="26" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B142" s="37" t="s">
         <v>75</v>
@@ -8550,13 +8562,13 @@
         <v>89</v>
       </c>
       <c r="D142" s="29" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="E142" s="28" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="F142" s="28" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="G142" s="30" t="s">
         <v>134</v>
@@ -8566,12 +8578,12 @@
       </c>
       <c r="I142" s="32"/>
       <c r="J142" s="33" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="26" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="B143" s="37" t="s">
         <v>75</v>
@@ -8580,13 +8592,13 @@
         <v>89</v>
       </c>
       <c r="D143" s="29" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="E143" s="28" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="F143" s="28" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="G143" s="30" t="s">
         <v>93</v>
@@ -8596,27 +8608,27 @@
       </c>
       <c r="I143" s="32"/>
       <c r="J143" s="33" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="26" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="B144" s="37" t="s">
         <v>75</v>
       </c>
       <c r="C144" s="28" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="D144" s="29" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="E144" s="28" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="F144" s="28" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="G144" s="30" t="s">
         <v>93</v>
@@ -8626,12 +8638,12 @@
       </c>
       <c r="I144" s="32"/>
       <c r="J144" s="33" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="26" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="B145" s="37" t="s">
         <v>75</v>
@@ -8640,13 +8652,13 @@
         <v>141</v>
       </c>
       <c r="D145" s="29" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="E145" s="28" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="F145" s="28" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="G145" s="30" t="s">
         <v>93</v>
@@ -8656,12 +8668,12 @@
       </c>
       <c r="I145" s="32"/>
       <c r="J145" s="33" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="26" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="B146" s="37" t="s">
         <v>75</v>
@@ -8670,13 +8682,13 @@
         <v>141</v>
       </c>
       <c r="D146" s="29" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="E146" s="28" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="F146" s="28" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="G146" s="30" t="s">
         <v>134</v>
@@ -8686,12 +8698,12 @@
       </c>
       <c r="I146" s="32"/>
       <c r="J146" s="33" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="26" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="B147" s="37" t="s">
         <v>75</v>
@@ -8700,13 +8712,13 @@
         <v>89</v>
       </c>
       <c r="D147" s="29" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="E147" s="28" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="F147" s="28" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="G147" s="30" t="s">
         <v>134</v>
@@ -8716,7 +8728,7 @@
       </c>
       <c r="I147" s="32"/>
       <c r="J147" s="33" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -8734,12 +8746,12 @@
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>"Chờ thử lại"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
       <formula>"Bỏ qua"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G300">
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
       <formula>"Cao"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>